<commit_message>
SEO 27/09: links da colecao Rheem e Rheem tankless para Rheem 40 gallon
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UPWTXrstC2Sqk1zwCfCnhH
</commit_message>
<xml_diff>
--- a/seo_2709_colecoes_Smart_Collections_IMPORTAR.xlsx
+++ b/seo_2709_colecoes_Smart_Collections_IMPORTAR.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -742,6 +742,70 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>rheem-manufacturing</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>UPDATE</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Rheem Manufacturing</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Rheem water heating: residential gas and electric tanks, gas and electric tankless, commercial electric and gas, point-of-use heaters, heat pump models, plus elements, conversion kits, anode rods and replacement parts.&lt;/p&gt;&lt;p&gt;Rheem's residential range spans atmospheric, direct vent, power direct vent and condensing. That vent classification is the decision that governs a replacement: an atmospheric unit draws combustion air from the room and vents by natural draft, while a direct-vent unit brings air in and exhaust out through a sealed pipe. Swapping between them means new venting, and often new combustion-air provision.&lt;/p&gt;&lt;p&gt;Warranty length is the shorthand for build quality across the line — 3, 6, 8 and 12 year models differ mainly in anode mass and tank lining, not in the burner. A 12-year tank in hard water can still be outlasted by a 6-year tank whose anode gets replaced.&lt;/p&gt;&lt;p&gt;Most residential connections are 3/4" MIP; commercial runs 1-1/2" and 2". Fuel types stocked include natural gas, propane, convertible and electric.&lt;/p&gt;&lt;p&gt;Shopping by type? See &lt;a href="/collections/rheem-40-gallon-water-heaters"&gt;Rheem 40 gallon water heaters&lt;/a&gt;, gas and electric, and &lt;a href="/collections/rheem-tankless-water-heaters"&gt;Rheem tankless water heaters&lt;/a&gt;.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Rheem Water Heaters &amp; Parts | The House Supplier</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Rheem residential and commercial water heaters: gas, electric, tankless, heat pump and point-of-use, plus elements, conversion kits and anode rods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>rheem-tankless-water-heaters</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>UPDATE</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Rheem Tankless Water Heaters</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;33 Rheem tankless units across four series, from the 18 kW electric RTEX at $651 to the 199,900 Btu/h IKONIC with a built-in recirculation pump at $2,505. Gas models run 120,000 to 199,900 Btu/h and deliver 3.3 to 5.6 GPM at a 70°F rise. Every gas unit takes 3/4" MIP on water and gas, holds 85 to 140°F, and modulates down to 11,000 Btu/h.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;The choice that decides the install cost is condensing or not.&lt;/strong&gt; The RTG series is non-condensing: 0.81 to 0.82 UEF, a copper fin heat exchanger, and exhaust hot enough to require 3"/5" stainless concentric venting. The RTGH series condenses: 0.93 UEF, copper and stainless, and exhaust cool enough to vent through 2" or 3" PVC, CPVC or polypropylene. The condensing unit often costs more on the invoice and less on the wall, because the vent material is a fraction of the price. Run both numbers before you pick.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;IKONIC is the top tier.&lt;/strong&gt; The RTGH-S models carry a full stainless heat exchanger, 0.96 UEF, a 15-year exchanger warranty instead of 12, and an elevation rating of 10,200 feet against 8,400 for the rest. The SR variants add a factory recirculation pump, which removes the cost of a separate pump and crossover valve on a retrofit.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Outdoor models need no vent at all.&lt;/strong&gt; The XL suffix is outdoor, DV is indoor direct vent. In a mild climate the outdoor unit deletes the entire venting line item.&lt;/p&gt;&lt;p&gt;Two things to check before ordering. Size the gas supply to the load, not to the connection: the 3/4" inlet is the fitting, and a 199,000 Btu/h unit on an undersized run will fault under demand. And on electric, read the amperage before the kilowatts: the RTEX-36 draws 150 A and wants four 40 A breakers, which most residential panels cannot give up.&lt;/p&gt;&lt;p&gt;Repair parts, vent kits, valve kits and recirculation components for these units are stocked separately.&lt;/p&gt;&lt;p&gt;Replacing a tank with a tank instead? See &lt;a href="/collections/rheem-40-gallon-water-heaters"&gt;Rheem 40 gallon water heaters&lt;/a&gt;, gas and electric.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Rheem Tankless Water Heaters | Gas &amp; Electric | The House Supplier</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Rheem RTG, RTGH and IKONIC gas tankless water heaters, 120,000-199,900 Btu/h, plus RTEX electric. Condensing and non-condensing, indoor and outdoor.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>